<commit_message>
feat: Atualiza o cálculo de "MEDIÇÕES ACUMULADAS", "SALDO DO CONTRATO" e "% EXEC." para usar valores diretos da fonte ANALITICA.xlsx.
</commit_message>
<xml_diff>
--- a/MEDIÇÕES_CONSOLIDADO.xlsx
+++ b/MEDIÇÕES_CONSOLIDADO.xlsx
@@ -1103,10 +1103,10 @@
         <v>0</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>31106158.75</v>
+        <v>36782151.81</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>0.8456862151698025</v>
+        <v>0.8456999999999999</v>
       </c>
       <c r="Q2" s="7" t="n">
         <v>5675993.06</v>
@@ -1386,13 +1386,13 @@
         <v>0</v>
       </c>
       <c r="O3" s="7" t="n">
-        <v>16018051.24</v>
+        <v>31022838.12</v>
       </c>
       <c r="P3" s="9" t="n">
-        <v>0.5163309423219207</v>
+        <v>0.5163</v>
       </c>
       <c r="Q3" s="7" t="n">
-        <v>15004786.88</v>
+        <v>15004786.89</v>
       </c>
       <c r="R3" s="7" t="n">
         <v>0</v>
@@ -1669,13 +1669,13 @@
         <v>0</v>
       </c>
       <c r="O4" s="7" t="n">
-        <v>13076583.13</v>
+        <v>51119038.92</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>0.2558065137035248</v>
+        <v>0.2558</v>
       </c>
       <c r="Q4" s="7" t="n">
-        <v>38042455.79</v>
+        <v>38042440.77</v>
       </c>
       <c r="R4" s="7" t="n">
         <v>0</v>
@@ -1952,10 +1952,10 @@
         <v>1122659.32</v>
       </c>
       <c r="O5" s="7" t="n">
-        <v>3806174.66</v>
+        <v>18990162.94</v>
       </c>
       <c r="P5" s="9" t="n">
-        <v>0.2004287520873689</v>
+        <v>0.2004</v>
       </c>
       <c r="Q5" s="7" t="n">
         <v>15183988.28</v>
@@ -2235,10 +2235,10 @@
         <v>0</v>
       </c>
       <c r="O6" s="7" t="n">
-        <v>7322834.12</v>
+        <v>8463890.939999999</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.8651853115678262</v>
+        <v>0.8652</v>
       </c>
       <c r="Q6" s="7" t="n">
         <v>1141056.82</v>
@@ -2518,10 +2518,10 @@
         <v>0</v>
       </c>
       <c r="O7" s="7" t="n">
-        <v>1222003.41</v>
+        <v>1528883.61</v>
       </c>
       <c r="P7" s="9" t="n">
-        <v>0.799278245909118</v>
+        <v>0.7993000000000001</v>
       </c>
       <c r="Q7" s="7" t="n">
         <v>306880.2</v>
@@ -2801,10 +2801,10 @@
         <v>0</v>
       </c>
       <c r="O8" s="7" t="n">
-        <v>1038880.21</v>
+        <v>3294597.99</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0.3153283687883267</v>
+        <v>0.3153</v>
       </c>
       <c r="Q8" s="7" t="n">
         <v>2255717.78</v>
@@ -3084,10 +3084,10 @@
         <v>1602190.92</v>
       </c>
       <c r="O9" s="7" t="n">
-        <v>27948056.39</v>
+        <v>62211091.02</v>
       </c>
       <c r="P9" s="9" t="n">
-        <v>0.4492455594616576</v>
+        <v>0.4492</v>
       </c>
       <c r="Q9" s="7" t="n">
         <v>34263034.63</v>
@@ -3367,10 +3367,10 @@
         <v>294296.16</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>54809333.5</v>
+        <v>56189486.28</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>0.9754375262816516</v>
+        <v>0.9754</v>
       </c>
       <c r="Q10" s="7" t="n">
         <v>1380152.78</v>
@@ -3650,10 +3650,10 @@
         <v>63006.28</v>
       </c>
       <c r="O11" s="7" t="n">
-        <v>63006.28</v>
+        <v>4705907.3</v>
       </c>
       <c r="P11" s="9" t="n">
-        <v>0.01338876352281737</v>
+        <v>0.0134</v>
       </c>
       <c r="Q11" s="7" t="n">
         <v>4642901.02</v>
@@ -3933,10 +3933,10 @@
         <v>0</v>
       </c>
       <c r="O12" s="7" t="n">
-        <v>1739254.2</v>
+        <v>2860442.12</v>
       </c>
       <c r="P12" s="9" t="n">
-        <v>0.6080368443183182</v>
+        <v>0.608</v>
       </c>
       <c r="Q12" s="7" t="n">
         <v>1121187.92</v>
@@ -4212,7 +4212,7 @@
         <v>0</v>
       </c>
       <c r="O13" s="7" t="n">
-        <v>0</v>
+        <v>5054505.24</v>
       </c>
       <c r="P13" s="9" t="n">
         <v>0</v>
@@ -4495,13 +4495,13 @@
         <v>1284711.9</v>
       </c>
       <c r="O14" s="7" t="n">
-        <v>2127588.26</v>
+        <v>7848019.53</v>
       </c>
       <c r="P14" s="9" t="n">
-        <v>0.271098746870728</v>
+        <v>0.1637</v>
       </c>
       <c r="Q14" s="7" t="n">
-        <v>5720431.27</v>
+        <v>6563307.63</v>
       </c>
       <c r="R14" s="7" t="n">
         <v>0</v>
@@ -4778,10 +4778,10 @@
         <v>0</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>32294745.04</v>
+        <v>48872552.26</v>
       </c>
       <c r="P15" s="9" t="n">
-        <v>0.6607951405564674</v>
+        <v>0.6607999999999999</v>
       </c>
       <c r="Q15" s="7" t="n">
         <v>16577807.22</v>
@@ -5061,7 +5061,7 @@
         <v>0</v>
       </c>
       <c r="O16" s="7" t="n">
-        <v>0</v>
+        <v>1302281.25</v>
       </c>
       <c r="P16" s="9" t="n">
         <v>0</v>
@@ -5344,13 +5344,13 @@
         <v>0</v>
       </c>
       <c r="O17" s="7" t="n">
-        <v>29783885.44</v>
+        <v>34662990.03</v>
       </c>
       <c r="P17" s="9" t="n">
-        <v>0.85924166998354</v>
+        <v>0.8592</v>
       </c>
       <c r="Q17" s="7" t="n">
-        <v>4879104.59</v>
+        <v>4879112.73</v>
       </c>
       <c r="R17" s="7" t="n">
         <v>0</v>
@@ -5627,10 +5627,10 @@
         <v>0</v>
       </c>
       <c r="O18" s="7" t="n">
-        <v>122778.19</v>
+        <v>7430869.32</v>
       </c>
       <c r="P18" s="9" t="n">
-        <v>0.01652272227013138</v>
+        <v>0.0165</v>
       </c>
       <c r="Q18" s="7" t="n">
         <v>7308091.13</v>
@@ -5910,10 +5910,10 @@
         <v>0</v>
       </c>
       <c r="O19" s="7" t="n">
-        <v>20145177.51</v>
+        <v>65678550.13</v>
       </c>
       <c r="P19" s="9" t="n">
-        <v>0.3067238462195937</v>
+        <v>0.3067</v>
       </c>
       <c r="Q19" s="7" t="n">
         <v>45533372.62</v>
@@ -6193,13 +6193,13 @@
         <v>0</v>
       </c>
       <c r="O20" s="7" t="n">
-        <v>22442987.52</v>
+        <v>58032411.71</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>0.3867319461433424</v>
+        <v>0.3867</v>
       </c>
       <c r="Q20" s="7" t="n">
-        <v>35589424.19</v>
+        <v>35589424.18</v>
       </c>
       <c r="R20" s="7" t="n">
         <v>0</v>
@@ -6476,10 +6476,10 @@
         <v>0</v>
       </c>
       <c r="O21" s="7" t="n">
-        <v>2045374.39</v>
+        <v>54283415</v>
       </c>
       <c r="P21" s="9" t="n">
-        <v>0.037679545216527</v>
+        <v>0.0377</v>
       </c>
       <c r="Q21" s="7" t="n">
         <v>52238040.61</v>
@@ -6759,13 +6759,13 @@
         <v>0</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>35796161.91</v>
+        <v>45862409.69</v>
       </c>
       <c r="P22" s="9" t="n">
-        <v>0.7805120174007151</v>
+        <v>0.7805</v>
       </c>
       <c r="Q22" s="7" t="n">
-        <v>10066247.78</v>
+        <v>10066247.71</v>
       </c>
       <c r="R22" s="7" t="n">
         <v>0</v>
@@ -7042,10 +7042,10 @@
         <v>0</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>3584685.32</v>
+        <v>6016602.48</v>
       </c>
       <c r="P23" s="9" t="n">
-        <v>0.5957989300300258</v>
+        <v>0.5958</v>
       </c>
       <c r="Q23" s="7" t="n">
         <v>2431917.16</v>
@@ -7325,13 +7325,13 @@
         <v>0</v>
       </c>
       <c r="O24" s="7" t="n">
-        <v>45451420.48</v>
+        <v>51414775.09</v>
       </c>
       <c r="P24" s="9" t="n">
-        <v>0.8840147681369541</v>
+        <v>0.8996</v>
       </c>
       <c r="Q24" s="7" t="n">
-        <v>5963354.61</v>
+        <v>5160639.5</v>
       </c>
       <c r="R24" s="7" t="n">
         <v>0</v>
@@ -7608,13 +7608,13 @@
         <v>0</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>2286082.54</v>
+        <v>2601911.32</v>
       </c>
       <c r="P25" s="9" t="n">
-        <v>0.8786166240285238</v>
+        <v>0.8786</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>315828.78</v>
+        <v>315830.9</v>
       </c>
       <c r="R25" s="7" t="n">
         <v>0</v>
@@ -7891,10 +7891,10 @@
         <v>0</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>425261.4</v>
+        <v>544550.48</v>
       </c>
       <c r="P26" s="9" t="n">
-        <v>0.7809402720570552</v>
+        <v>0.7809</v>
       </c>
       <c r="Q26" s="7" t="n">
         <v>119289.08</v>
@@ -8174,13 +8174,13 @@
         <v>0</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>19844966.53</v>
+        <v>28459856.91</v>
       </c>
       <c r="P27" s="9" t="n">
-        <v>0.697296778151651</v>
+        <v>0.6973</v>
       </c>
       <c r="Q27" s="7" t="n">
-        <v>8614890.380000001</v>
+        <v>8614890.33</v>
       </c>
       <c r="R27" s="7" t="n">
         <v>0</v>
@@ -8457,10 +8457,10 @@
         <v>0</v>
       </c>
       <c r="O28" s="7" t="n">
-        <v>42048979.52</v>
+        <v>43796954.98</v>
       </c>
       <c r="P28" s="9" t="n">
-        <v>0.9600891098297082</v>
+        <v>0.9601000000000001</v>
       </c>
       <c r="Q28" s="7" t="n">
         <v>1747975.46</v>
@@ -8740,10 +8740,10 @@
         <v>499862.54</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>36377601.26</v>
+        <v>45726170.25</v>
       </c>
       <c r="P29" s="9" t="n">
-        <v>0.7955532042397536</v>
+        <v>0.7956</v>
       </c>
       <c r="Q29" s="7" t="n">
         <v>9348568.99</v>
@@ -9023,13 +9023,13 @@
         <v>0</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>13115141.03</v>
+        <v>22825141.32</v>
       </c>
       <c r="P30" s="9" t="n">
-        <v>0.574591887346089</v>
+        <v>0.5746</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>9710000.289999999</v>
+        <v>9709999.51</v>
       </c>
       <c r="R30" s="7" t="n">
         <v>0</v>
@@ -9306,10 +9306,10 @@
         <v>0</v>
       </c>
       <c r="O31" s="7" t="n">
-        <v>14348711.09</v>
+        <v>26504288.68</v>
       </c>
       <c r="P31" s="9" t="n">
-        <v>0.5413731816476728</v>
+        <v>0.5414</v>
       </c>
       <c r="Q31" s="7" t="n">
         <v>12155577.59</v>
@@ -9589,10 +9589,10 @@
         <v>3545422.68</v>
       </c>
       <c r="O32" s="7" t="n">
-        <v>19434508.22</v>
+        <v>20106028.53</v>
       </c>
       <c r="P32" s="9" t="n">
-        <v>0.9666010465966449</v>
+        <v>0.9666</v>
       </c>
       <c r="Q32" s="7" t="n">
         <v>671520.3100000001</v>
@@ -9872,13 +9872,13 @@
         <v>0</v>
       </c>
       <c r="O33" s="7" t="n">
-        <v>7571952.28</v>
+        <v>7795660.46</v>
       </c>
       <c r="P33" s="9" t="n">
-        <v>0.971303498767313</v>
+        <v>0.9712999999999999</v>
       </c>
       <c r="Q33" s="7" t="n">
-        <v>223708.18</v>
+        <v>223708.17</v>
       </c>
       <c r="R33" s="7" t="n">
         <v>0</v>
@@ -10155,7 +10155,7 @@
         <v>0</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>0</v>
+        <v>41522873.42</v>
       </c>
       <c r="P34" s="9" t="n">
         <v>0</v>
@@ -10438,10 +10438,10 @@
         <v>1285251.84</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>5666949.72</v>
+        <v>7066834.9</v>
       </c>
       <c r="P35" s="9" t="n">
-        <v>0.80190775646959</v>
+        <v>0.8018999999999999</v>
       </c>
       <c r="Q35" s="7" t="n">
         <v>1399885.18</v>
@@ -10721,10 +10721,10 @@
         <v>3055826.41</v>
       </c>
       <c r="O36" s="7" t="n">
-        <v>5476795.79</v>
+        <v>10349390.52</v>
       </c>
       <c r="P36" s="9" t="n">
-        <v>0.5291901759254515</v>
+        <v>0.5292</v>
       </c>
       <c r="Q36" s="7" t="n">
         <v>4872594.73</v>
@@ -11004,10 +11004,10 @@
         <v>7440875.08</v>
       </c>
       <c r="O37" s="7" t="n">
-        <v>21232327.94</v>
+        <v>27434724</v>
       </c>
       <c r="P37" s="9" t="n">
-        <v>0.7739216891702646</v>
+        <v>0.7739</v>
       </c>
       <c r="Q37" s="7" t="n">
         <v>6202396.06</v>
@@ -11287,10 +11287,10 @@
         <v>137056.25</v>
       </c>
       <c r="O38" s="7" t="n">
-        <v>685145.5600000001</v>
+        <v>763285.0699999999</v>
       </c>
       <c r="P38" s="9" t="n">
-        <v>0.8976273569716227</v>
+        <v>0.8976000000000001</v>
       </c>
       <c r="Q38" s="7" t="n">
         <v>78139.50999999999</v>
@@ -11570,10 +11570,10 @@
         <v>0</v>
       </c>
       <c r="O39" s="7" t="n">
-        <v>164482.69</v>
+        <v>256613.37</v>
       </c>
       <c r="P39" s="9" t="n">
-        <v>0.6409747473407174</v>
+        <v>0.6409999999999999</v>
       </c>
       <c r="Q39" s="7" t="n">
         <v>92130.67999999999</v>
@@ -11853,7 +11853,7 @@
         <v>0</v>
       </c>
       <c r="O40" s="7" t="n">
-        <v>0</v>
+        <v>2742607.66</v>
       </c>
       <c r="P40" s="9" t="n">
         <v>0</v>
@@ -12136,13 +12136,13 @@
         <v>0</v>
       </c>
       <c r="O41" s="7" t="n">
-        <v>2301268.72</v>
+        <v>15203482.79</v>
       </c>
       <c r="P41" s="9" t="n">
-        <v>0.1513645755901172</v>
+        <v>0.15</v>
       </c>
       <c r="Q41" s="7" t="n">
-        <v>12902214.07</v>
+        <v>12923552.74</v>
       </c>
       <c r="R41" s="7" t="n">
         <v>0</v>
@@ -12419,13 +12419,13 @@
         <v>3468001.87</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>14615806.68</v>
+        <v>24187461.93</v>
       </c>
       <c r="P42" s="9" t="n">
-        <v>0.6042720283053692</v>
+        <v>0.6042999999999999</v>
       </c>
       <c r="Q42" s="7" t="n">
-        <v>9571655.25</v>
+        <v>9571655.24</v>
       </c>
       <c r="R42" s="7" t="n">
         <v>0</v>
@@ -12702,10 +12702,10 @@
         <v>0</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>10511270.47</v>
+        <v>12432476.25</v>
       </c>
       <c r="P43" s="9" t="n">
-        <v>0.8454687753777129</v>
+        <v>0.8454999999999999</v>
       </c>
       <c r="Q43" s="7" t="n">
         <v>1921205.78</v>
@@ -12985,10 +12985,10 @@
         <v>0</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>10301084.52</v>
+        <v>12100122.6</v>
       </c>
       <c r="P44" s="9" t="n">
-        <v>0.851320673395491</v>
+        <v>0.8512999999999999</v>
       </c>
       <c r="Q44" s="7" t="n">
         <v>1799038.08</v>
@@ -13268,13 +13268,13 @@
         <v>0</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>56075179.54</v>
+        <v>59148617.81</v>
       </c>
       <c r="P45" s="9" t="n">
-        <v>0.9480387136032045</v>
+        <v>0.948</v>
       </c>
       <c r="Q45" s="7" t="n">
-        <v>3073438.27</v>
+        <v>3073439.17</v>
       </c>
       <c r="R45" s="7" t="n">
         <v>0</v>
@@ -13551,10 +13551,10 @@
         <v>0</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>22022321.06</v>
+        <v>116500000</v>
       </c>
       <c r="P46" s="9" t="n">
-        <v>0.1890327987982832</v>
+        <v>0.189</v>
       </c>
       <c r="Q46" s="7" t="n">
         <v>94477678.94</v>
@@ -13834,10 +13834,10 @@
         <v>0</v>
       </c>
       <c r="O47" s="7" t="n">
-        <v>38738669.02</v>
+        <v>41651255.98</v>
       </c>
       <c r="P47" s="9" t="n">
-        <v>0.9300720496544316</v>
+        <v>0.9301</v>
       </c>
       <c r="Q47" s="7" t="n">
         <v>2912586.96</v>
@@ -14117,10 +14117,10 @@
         <v>0</v>
       </c>
       <c r="O48" s="7" t="n">
-        <v>54247297.54</v>
+        <v>104939756.55</v>
       </c>
       <c r="P48" s="9" t="n">
-        <v>0.5169375203777334</v>
+        <v>0.5169</v>
       </c>
       <c r="Q48" s="7" t="n">
         <v>50692459.01</v>
@@ -14400,10 +14400,10 @@
         <v>1537890.45</v>
       </c>
       <c r="O49" s="7" t="n">
-        <v>63449041.49</v>
+        <v>74609626.42</v>
       </c>
       <c r="P49" s="9" t="n">
-        <v>0.8504136065877919</v>
+        <v>0.8504</v>
       </c>
       <c r="Q49" s="7" t="n">
         <v>11160584.93</v>
@@ -15242,10 +15242,10 @@
         <v>0</v>
       </c>
       <c r="P2" s="7" t="n">
-        <v>1088826.01</v>
+        <v>1212482.21</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>0.8980140087993539</v>
+        <v>0.898</v>
       </c>
       <c r="R2" s="7" t="n">
         <v>123656.2</v>
@@ -15522,13 +15522,13 @@
         <v>0</v>
       </c>
       <c r="P3" s="7" t="n">
-        <v>32682339.39</v>
+        <v>69450000</v>
       </c>
       <c r="Q3" s="9" t="n">
-        <v>0.4705880401727862</v>
+        <v>0.4456</v>
       </c>
       <c r="R3" s="7" t="n">
-        <v>36767660.61</v>
+        <v>38500569.52</v>
       </c>
       <c r="S3" s="7" t="n">
         <v>0</v>
@@ -15802,13 +15802,13 @@
         <v>0</v>
       </c>
       <c r="P4" s="7" t="n">
-        <v>75957961.34</v>
+        <v>84484346.70999999</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.8990773356007883</v>
+        <v>0.4495</v>
       </c>
       <c r="R4" s="7" t="n">
-        <v>8526385.369999999</v>
+        <v>46505366.04</v>
       </c>
       <c r="S4" s="7" t="n">
         <v>0</v>
@@ -16090,13 +16090,13 @@
         <v>0</v>
       </c>
       <c r="P5" s="7" t="n">
-        <v>1127526.06</v>
+        <v>2069000</v>
       </c>
       <c r="Q5" s="9" t="n">
-        <v>0.5449618463025616</v>
+        <v>0.545</v>
       </c>
       <c r="R5" s="7" t="n">
-        <v>941473.9399999999</v>
+        <v>941483.9399999999</v>
       </c>
       <c r="S5" s="7" t="n">
         <v>0</v>
@@ -16373,7 +16373,7 @@
         <v>6948720.19</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.9999999999999999</v>
+        <v>1</v>
       </c>
       <c r="R6" s="7" t="n">
         <v>0</v>
@@ -16930,10 +16930,10 @@
         <v>0</v>
       </c>
       <c r="P8" s="7" t="n">
-        <v>6743573.85</v>
+        <v>6743574.04</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>0.9999999718250295</v>
+        <v>1</v>
       </c>
       <c r="R8" s="7" t="n">
         <v>0.19</v>
@@ -17214,13 +17214,13 @@
         <v>0</v>
       </c>
       <c r="P9" s="7" t="n">
-        <v>8394719</v>
+        <v>8396309.76</v>
       </c>
       <c r="Q9" s="9" t="n">
-        <v>0.9998105405772927</v>
+        <v>0.9998</v>
       </c>
       <c r="R9" s="7" t="n">
-        <v>1590.76</v>
+        <v>1540.74</v>
       </c>
       <c r="S9" s="7" t="n">
         <v>0</v>
@@ -17498,13 +17498,13 @@
         <v>0</v>
       </c>
       <c r="P10" s="7" t="n">
-        <v>4374443.73</v>
+        <v>4374443.78</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>0.9999999885699754</v>
+        <v>1</v>
       </c>
       <c r="R10" s="7" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="S10" s="7" t="n">
         <v>0</v>
@@ -17786,10 +17786,10 @@
         <v>0</v>
       </c>
       <c r="P11" s="7" t="n">
-        <v>1740561.74</v>
+        <v>1741703.69</v>
       </c>
       <c r="Q11" s="9" t="n">
-        <v>0.9993443488656789</v>
+        <v>0.9993000000000001</v>
       </c>
       <c r="R11" s="7" t="n">
         <v>1141.95</v>
@@ -18070,10 +18070,10 @@
         <v>0</v>
       </c>
       <c r="P12" s="7" t="n">
-        <v>7104640.05</v>
+        <v>8811881.779999999</v>
       </c>
       <c r="Q12" s="9" t="n">
-        <v>0.806256850395467</v>
+        <v>0.8062999999999999</v>
       </c>
       <c r="R12" s="7" t="n">
         <v>1707241.73</v>
@@ -18350,10 +18350,10 @@
         <v>0</v>
       </c>
       <c r="P13" s="7" t="n">
-        <v>1285178.36</v>
+        <v>1332580.86</v>
       </c>
       <c r="Q13" s="9" t="n">
-        <v>0.9644280497920404</v>
+        <v>0.9643999999999999</v>
       </c>
       <c r="R13" s="7" t="n">
         <v>47402.5</v>
@@ -18634,13 +18634,13 @@
         <v>0</v>
       </c>
       <c r="P14" s="7" t="n">
-        <v>5132338.31</v>
+        <v>5272095.08</v>
       </c>
       <c r="Q14" s="9" t="n">
-        <v>0.9734912273243751</v>
+        <v>0.9998999999999999</v>
       </c>
       <c r="R14" s="7" t="n">
-        <v>139756.77</v>
+        <v>401.87</v>
       </c>
       <c r="S14" s="7" t="n">
         <v>0</v>
@@ -18914,10 +18914,10 @@
         <v>0</v>
       </c>
       <c r="P15" s="7" t="n">
-        <v>3607318.65</v>
+        <v>3607367.42</v>
       </c>
       <c r="Q15" s="9" t="n">
-        <v>0.999986480445621</v>
+        <v>1</v>
       </c>
       <c r="R15" s="7" t="n">
         <v>48.77</v>
@@ -19198,10 +19198,10 @@
         <v>0</v>
       </c>
       <c r="P16" s="7" t="n">
-        <v>4625557.49</v>
+        <v>4645152.25</v>
       </c>
       <c r="Q16" s="9" t="n">
-        <v>0.9957816754014897</v>
+        <v>0.9958</v>
       </c>
       <c r="R16" s="7" t="n">
         <v>19594.76</v>
@@ -19482,13 +19482,13 @@
         <v>0</v>
       </c>
       <c r="P17" s="7" t="n">
-        <v>10939879.36</v>
+        <v>11046611.98</v>
       </c>
       <c r="Q17" s="9" t="n">
-        <v>0.9903379769115415</v>
+        <v>0.9903</v>
       </c>
       <c r="R17" s="7" t="n">
-        <v>106732.62</v>
+        <v>106732.59</v>
       </c>
       <c r="S17" s="7" t="n">
         <v>0</v>
@@ -19762,7 +19762,7 @@
         <v>0</v>
       </c>
       <c r="P18" s="7" t="n">
-        <v>0</v>
+        <v>1305890.95</v>
       </c>
       <c r="Q18" s="9" t="n">
         <v>0</v>
@@ -20046,13 +20046,13 @@
         <v>0</v>
       </c>
       <c r="P19" s="7" t="n">
-        <v>6171355.17</v>
+        <v>30334596.91</v>
       </c>
       <c r="Q19" s="9" t="n">
-        <v>0.2034427946515937</v>
+        <v>0.2034</v>
       </c>
       <c r="R19" s="7" t="n">
-        <v>24163241.74</v>
+        <v>24163359.13</v>
       </c>
       <c r="S19" s="7" t="n">
         <v>0</v>
@@ -20330,13 +20330,13 @@
         <v>0</v>
       </c>
       <c r="P20" s="7" t="n">
-        <v>10061305.06</v>
+        <v>10061005.41</v>
       </c>
       <c r="Q20" s="9" t="n">
-        <v>1.000029783305722</v>
+        <v>1</v>
       </c>
       <c r="R20" s="7" t="n">
-        <v>-299.65</v>
+        <v>0.02</v>
       </c>
       <c r="S20" s="7" t="n">
         <v>0</v>
@@ -20618,10 +20618,10 @@
         <v>0</v>
       </c>
       <c r="P21" s="7" t="n">
-        <v>32314427.7</v>
+        <v>32464769.58</v>
       </c>
       <c r="Q21" s="9" t="n">
-        <v>0.9953690760185584</v>
+        <v>0.9954000000000001</v>
       </c>
       <c r="R21" s="7" t="n">
         <v>150341.88</v>
@@ -20902,13 +20902,13 @@
         <v>0</v>
       </c>
       <c r="P22" s="7" t="n">
-        <v>17677149.64</v>
+        <v>17695067.23</v>
       </c>
       <c r="Q22" s="9" t="n">
-        <v>0.9989874245874792</v>
+        <v>0.9990000000000001</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>17917.59</v>
+        <v>17917.39</v>
       </c>
       <c r="S22" s="7" t="n">
         <v>0</v>
@@ -21462,13 +21462,13 @@
         <v>0</v>
       </c>
       <c r="P24" s="7" t="n">
-        <v>30651574.56</v>
+        <v>68148567.14</v>
       </c>
       <c r="Q24" s="9" t="n">
-        <v>0.4497757744052255</v>
+        <v>0.4476</v>
       </c>
       <c r="R24" s="7" t="n">
-        <v>37496992.58</v>
+        <v>37645831.73</v>
       </c>
       <c r="S24" s="7" t="n">
         <v>0</v>
@@ -21746,10 +21746,10 @@
         <v>0</v>
       </c>
       <c r="P25" s="7" t="n">
-        <v>133579.45</v>
+        <v>47996411.38</v>
       </c>
       <c r="Q25" s="9" t="n">
-        <v>0.002783113281999709</v>
+        <v>0.0028</v>
       </c>
       <c r="R25" s="7" t="n">
         <v>47862831.93</v>
@@ -22034,10 +22034,10 @@
         <v>0</v>
       </c>
       <c r="P26" s="7" t="n">
-        <v>19406169.39</v>
+        <v>19451386.88</v>
       </c>
       <c r="Q26" s="9" t="n">
-        <v>0.9976753590744477</v>
+        <v>0.9976999999999999</v>
       </c>
       <c r="R26" s="7" t="n">
         <v>45217.49</v>
@@ -22318,13 +22318,13 @@
         <v>0</v>
       </c>
       <c r="P27" s="7" t="n">
-        <v>28044628.65</v>
+        <v>30543662.31</v>
       </c>
       <c r="Q27" s="9" t="n">
-        <v>0.9181815973920777</v>
+        <v>0.9181999999999999</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>2499033.66</v>
+        <v>2499033.71</v>
       </c>
       <c r="S27" s="7" t="n">
         <v>0</v>
@@ -22598,13 +22598,13 @@
         <v>0</v>
       </c>
       <c r="P28" s="7" t="n">
-        <v>5450476.84</v>
+        <v>5978542.15</v>
       </c>
       <c r="Q28" s="9" t="n">
-        <v>0.9116732312408299</v>
+        <v>0.9117000000000001</v>
       </c>
       <c r="R28" s="7" t="n">
-        <v>528065.3100000001</v>
+        <v>528065.11</v>
       </c>
       <c r="S28" s="7" t="n">
         <v>0</v>
@@ -22872,7 +22872,7 @@
         <v>0</v>
       </c>
       <c r="P29" s="7" t="n">
-        <v>0</v>
+        <v>11620104.78</v>
       </c>
       <c r="Q29" s="9" t="n">
         <v>0</v>
@@ -23156,13 +23156,13 @@
         <v>0</v>
       </c>
       <c r="P30" s="7" t="n">
-        <v>4324004.79</v>
+        <v>4444784.22</v>
       </c>
       <c r="Q30" s="9" t="n">
-        <v>0.9728267056347676</v>
+        <v>0.9728</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>120779.43</v>
+        <v>120779.41</v>
       </c>
       <c r="S30" s="7" t="n">
         <v>0</v>
@@ -23444,10 +23444,10 @@
         <v>0</v>
       </c>
       <c r="P31" s="7" t="n">
-        <v>2226331.45</v>
+        <v>2755604.93</v>
       </c>
       <c r="Q31" s="9" t="n">
-        <v>0.8079283883412126</v>
+        <v>0.8079000000000001</v>
       </c>
       <c r="R31" s="7" t="n">
         <v>529273.48</v>
@@ -23724,7 +23724,7 @@
         <v>0</v>
       </c>
       <c r="P32" s="7" t="n">
-        <v>0</v>
+        <v>1712576.84</v>
       </c>
       <c r="Q32" s="9" t="n">
         <v>0</v>
@@ -24008,13 +24008,13 @@
         <v>0</v>
       </c>
       <c r="P33" s="7" t="n">
-        <v>56408430.85</v>
+        <v>58086688.76</v>
       </c>
       <c r="Q33" s="9" t="n">
-        <v>0.971107702197759</v>
+        <v>0.9711</v>
       </c>
       <c r="R33" s="7" t="n">
-        <v>1678257.91</v>
+        <v>1678137.85</v>
       </c>
       <c r="S33" s="7" t="n">
         <v>0</v>
@@ -24282,10 +24282,10 @@
         <v>0</v>
       </c>
       <c r="P34" s="7" t="n">
-        <v>9021796.75</v>
+        <v>18996888.26</v>
       </c>
       <c r="Q34" s="9" t="n">
-        <v>0.4749091865216877</v>
+        <v>0.4749</v>
       </c>
       <c r="R34" s="7" t="n">
         <v>9975091.51</v>
@@ -24562,13 +24562,13 @@
         <v>0</v>
       </c>
       <c r="P35" s="7" t="n">
-        <v>9986334.550000001</v>
+        <v>11942741.09</v>
       </c>
       <c r="Q35" s="9" t="n">
-        <v>0.8361844634111548</v>
+        <v>0.8362000000000001</v>
       </c>
       <c r="R35" s="7" t="n">
-        <v>1956406.54</v>
+        <v>1956406.46</v>
       </c>
       <c r="S35" s="7" t="n">
         <v>0</v>
@@ -24842,10 +24842,10 @@
         <v>0</v>
       </c>
       <c r="P36" s="7" t="n">
-        <v>50454918.61</v>
+        <v>54913544.95</v>
       </c>
       <c r="Q36" s="9" t="n">
-        <v>0.9188064375727395</v>
+        <v>0.9188</v>
       </c>
       <c r="R36" s="7" t="n">
         <v>4458626.34</v>
@@ -25406,10 +25406,10 @@
         <v>0</v>
       </c>
       <c r="P38" s="7" t="n">
-        <v>9661616.369999999</v>
+        <v>9751616.369999999</v>
       </c>
       <c r="Q38" s="9" t="n">
-        <v>0.9907707608067029</v>
+        <v>0.9908</v>
       </c>
       <c r="R38" s="7" t="n">
         <v>90000</v>
@@ -25690,13 +25690,13 @@
         <v>0</v>
       </c>
       <c r="P39" s="7" t="n">
-        <v>13792679.65</v>
+        <v>13792679.79</v>
       </c>
       <c r="Q39" s="9" t="n">
-        <v>0.9999999898496883</v>
+        <v>1</v>
       </c>
       <c r="R39" s="7" t="n">
-        <v>0.14</v>
+        <v>0</v>
       </c>
       <c r="S39" s="7" t="n">
         <v>0</v>
@@ -25978,13 +25978,13 @@
         <v>0</v>
       </c>
       <c r="P40" s="7" t="n">
-        <v>6488132.93</v>
+        <v>7704834.91</v>
       </c>
       <c r="Q40" s="9" t="n">
-        <v>0.8420859117408395</v>
+        <v>0.8421</v>
       </c>
       <c r="R40" s="7" t="n">
-        <v>1216701.98</v>
+        <v>1216701.97</v>
       </c>
       <c r="S40" s="7" t="n">
         <v>0</v>
@@ -26258,13 +26258,13 @@
         <v>0</v>
       </c>
       <c r="P41" s="7" t="n">
-        <v>74305044.28</v>
+        <v>80552394.92</v>
       </c>
       <c r="Q41" s="9" t="n">
-        <v>0.9224436387496049</v>
+        <v>0.9224</v>
       </c>
       <c r="R41" s="7" t="n">
-        <v>6247350.64</v>
+        <v>6247349.45</v>
       </c>
       <c r="S41" s="7" t="n">
         <v>0</v>
@@ -26538,13 +26538,13 @@
         <v>0</v>
       </c>
       <c r="P42" s="7" t="n">
-        <v>6453162.33</v>
+        <v>6453162.72</v>
       </c>
       <c r="Q42" s="9" t="n">
-        <v>0.9999999395645179</v>
+        <v>1</v>
       </c>
       <c r="R42" s="7" t="n">
-        <v>0.39</v>
+        <v>0</v>
       </c>
       <c r="S42" s="7" t="n">
         <v>0</v>
@@ -26818,13 +26818,13 @@
         <v>0</v>
       </c>
       <c r="P43" s="7" t="n">
-        <v>25313733.13</v>
+        <v>37535912.65</v>
       </c>
       <c r="Q43" s="9" t="n">
-        <v>0.6743870427778181</v>
+        <v>0.6744</v>
       </c>
       <c r="R43" s="7" t="n">
-        <v>12222179.52</v>
+        <v>12222179.43</v>
       </c>
       <c r="S43" s="7" t="n">
         <v>0</v>
@@ -27102,10 +27102,10 @@
         <v>0</v>
       </c>
       <c r="P44" s="7" t="n">
-        <v>3034704.58</v>
+        <v>3107538.75</v>
       </c>
       <c r="Q44" s="9" t="n">
-        <v>0.9765621040123796</v>
+        <v>0.9765999999999999</v>
       </c>
       <c r="R44" s="7" t="n">
         <v>72834.17</v>
@@ -27386,10 +27386,10 @@
         <v>0</v>
       </c>
       <c r="P45" s="7" t="n">
-        <v>41562191.24</v>
+        <v>51359899.57</v>
       </c>
       <c r="Q45" s="9" t="n">
-        <v>0.8092342778699091</v>
+        <v>0.8092</v>
       </c>
       <c r="R45" s="7" t="n">
         <v>9797708.33</v>
@@ -27670,10 +27670,10 @@
         <v>0</v>
       </c>
       <c r="P46" s="7" t="n">
-        <v>13242495.84</v>
+        <v>13242425.64</v>
       </c>
       <c r="Q46" s="9" t="n">
-        <v>1.000005301143605</v>
+        <v>1</v>
       </c>
       <c r="R46" s="7" t="n">
         <v>-70.2</v>
@@ -27958,10 +27958,10 @@
         <v>0</v>
       </c>
       <c r="P47" s="7" t="n">
-        <v>6450491.31</v>
+        <v>7234583.77</v>
       </c>
       <c r="Q47" s="9" t="n">
-        <v>0.8916188567403928</v>
+        <v>0.8915999999999999</v>
       </c>
       <c r="R47" s="7" t="n">
         <v>784092.46</v>
@@ -28242,13 +28242,13 @@
         <v>0</v>
       </c>
       <c r="P48" s="7" t="n">
-        <v>11566431.39</v>
+        <v>12560309.12</v>
       </c>
       <c r="Q48" s="9" t="n">
-        <v>0.9208715549510299</v>
+        <v>0.9209000000000001</v>
       </c>
       <c r="R48" s="7" t="n">
-        <v>993877.73</v>
+        <v>993876.73</v>
       </c>
       <c r="S48" s="7" t="n">
         <v>0</v>
@@ -28526,13 +28526,13 @@
         <v>0</v>
       </c>
       <c r="P49" s="7" t="n">
-        <v>20500685.69</v>
+        <v>22472818</v>
       </c>
       <c r="Q49" s="9" t="n">
-        <v>0.9122436576489871</v>
+        <v>0.9122</v>
       </c>
       <c r="R49" s="7" t="n">
-        <v>1972132.31</v>
+        <v>1972132.32</v>
       </c>
       <c r="S49" s="7" t="n">
         <v>0</v>
@@ -28810,13 +28810,13 @@
         <v>0</v>
       </c>
       <c r="P50" s="7" t="n">
-        <v>43785880.08</v>
+        <v>45237596.81</v>
       </c>
       <c r="Q50" s="9" t="n">
-        <v>0.9679090660784375</v>
+        <v>0.9865</v>
       </c>
       <c r="R50" s="7" t="n">
-        <v>1451716.73</v>
+        <v>610868.61</v>
       </c>
       <c r="S50" s="7" t="n">
         <v>0</v>
@@ -29090,10 +29090,10 @@
         <v>0</v>
       </c>
       <c r="P51" s="7" t="n">
-        <v>133236.58</v>
+        <v>12679339.18</v>
       </c>
       <c r="Q51" s="9" t="n">
-        <v>0.01050816435371989</v>
+        <v>0.0105</v>
       </c>
       <c r="R51" s="7" t="n">
         <v>12546102.6</v>
@@ -29374,10 +29374,10 @@
         <v>0</v>
       </c>
       <c r="P52" s="7" t="n">
-        <v>33048630.33</v>
+        <v>34508101.15</v>
       </c>
       <c r="Q52" s="9" t="n">
-        <v>0.9577064291756896</v>
+        <v>0.9577</v>
       </c>
       <c r="R52" s="7" t="n">
         <v>1459470.82</v>
@@ -29658,13 +29658,13 @@
         <v>0</v>
       </c>
       <c r="P53" s="7" t="n">
-        <v>151308</v>
+        <v>11494433.26</v>
       </c>
       <c r="Q53" s="9" t="n">
-        <v>0.01316358941562988</v>
+        <v>0.0132</v>
       </c>
       <c r="R53" s="7" t="n">
-        <v>11343125.26</v>
+        <v>11343147.64</v>
       </c>
       <c r="S53" s="7" t="n">
         <v>0</v>
@@ -29942,10 +29942,10 @@
         <v>0</v>
       </c>
       <c r="P54" s="7" t="n">
-        <v>13332401.6</v>
+        <v>20185137.81</v>
       </c>
       <c r="Q54" s="9" t="n">
-        <v>0.6605058496749495</v>
+        <v>0.6605</v>
       </c>
       <c r="R54" s="7" t="n">
         <v>6852736.21</v>
@@ -30226,10 +30226,10 @@
         <v>0</v>
       </c>
       <c r="P55" s="7" t="n">
-        <v>12534756.7</v>
+        <v>30477728.43</v>
       </c>
       <c r="Q55" s="9" t="n">
-        <v>0.4112759495442489</v>
+        <v>0.4113</v>
       </c>
       <c r="R55" s="7" t="n">
         <v>17942971.73</v>
@@ -30514,13 +30514,13 @@
         <v>0</v>
       </c>
       <c r="P56" s="7" t="n">
-        <v>6523029.66</v>
+        <v>6478069.43</v>
       </c>
       <c r="Q56" s="9" t="n">
-        <v>1.006940374827073</v>
+        <v>1</v>
       </c>
       <c r="R56" s="7" t="n">
-        <v>-44960.23</v>
+        <v>39.99</v>
       </c>
       <c r="S56" s="7" t="n">
         <v>0</v>
@@ -30802,10 +30802,10 @@
         <v>0</v>
       </c>
       <c r="P57" s="7" t="n">
-        <v>6007931.02</v>
+        <v>6055289.34</v>
       </c>
       <c r="Q57" s="9" t="n">
-        <v>0.9921790161723304</v>
+        <v>0.9922</v>
       </c>
       <c r="R57" s="7" t="n">
         <v>47358.32</v>
@@ -31086,10 +31086,10 @@
         <v>0</v>
       </c>
       <c r="P58" s="7" t="n">
-        <v>5551029.21</v>
+        <v>5722613.87</v>
       </c>
       <c r="Q58" s="9" t="n">
-        <v>0.9700163834398283</v>
+        <v>0.97</v>
       </c>
       <c r="R58" s="7" t="n">
         <v>171584.66</v>
@@ -31374,13 +31374,13 @@
         <v>0</v>
       </c>
       <c r="P59" s="7" t="n">
-        <v>5580983.94</v>
+        <v>5581731.3</v>
       </c>
       <c r="Q59" s="9" t="n">
-        <v>0.9998661060592436</v>
+        <v>1</v>
       </c>
       <c r="R59" s="7" t="n">
-        <v>747.36</v>
+        <v>1</v>
       </c>
       <c r="S59" s="7" t="n">
         <v>0</v>
@@ -31658,10 +31658,10 @@
         <v>0</v>
       </c>
       <c r="P60" s="7" t="n">
-        <v>12032786.93</v>
+        <v>13208831.36</v>
       </c>
       <c r="Q60" s="9" t="n">
-        <v>0.9109652929962155</v>
+        <v>0.9109999999999999</v>
       </c>
       <c r="R60" s="7" t="n">
         <v>1176044.43</v>
@@ -31946,13 +31946,13 @@
         <v>0</v>
       </c>
       <c r="P61" s="7" t="n">
-        <v>111124067.68</v>
+        <v>113557951.65</v>
       </c>
       <c r="Q61" s="9" t="n">
-        <v>0.9785670317698092</v>
+        <v>0.9786</v>
       </c>
       <c r="R61" s="7" t="n">
-        <v>2433883.97</v>
+        <v>2424755.97</v>
       </c>
       <c r="S61" s="7" t="n">
         <v>0</v>
@@ -32234,10 +32234,10 @@
         <v>0</v>
       </c>
       <c r="P62" s="7" t="n">
-        <v>8552770.91</v>
+        <v>12950372.72</v>
       </c>
       <c r="Q62" s="9" t="n">
-        <v>0.6604266220686813</v>
+        <v>0.6604000000000001</v>
       </c>
       <c r="R62" s="7" t="n">
         <v>4397601.81</v>
@@ -32518,13 +32518,13 @@
         <v>0</v>
       </c>
       <c r="P63" s="7" t="n">
-        <v>20859058.41</v>
+        <v>20859068.44</v>
       </c>
       <c r="Q63" s="9" t="n">
-        <v>0.9999995191539819</v>
+        <v>1</v>
       </c>
       <c r="R63" s="7" t="n">
-        <v>10.03</v>
+        <v>0</v>
       </c>
       <c r="S63" s="7" t="n">
         <v>0</v>
@@ -32806,13 +32806,13 @@
         <v>0</v>
       </c>
       <c r="P64" s="7" t="n">
-        <v>81959611</v>
+        <v>81950979.23</v>
       </c>
       <c r="Q64" s="9" t="n">
-        <v>1.000105328454658</v>
+        <v>1</v>
       </c>
       <c r="R64" s="7" t="n">
-        <v>-8631.77</v>
+        <v>0.23</v>
       </c>
       <c r="S64" s="7" t="n">
         <v>0</v>
@@ -33086,10 +33086,10 @@
         <v>0</v>
       </c>
       <c r="P65" s="7" t="n">
-        <v>2042159.29</v>
+        <v>8973983.869999999</v>
       </c>
       <c r="Q65" s="9" t="n">
-        <v>0.2275644039016977</v>
+        <v>0.2276</v>
       </c>
       <c r="R65" s="7" t="n">
         <v>6931824.58</v>
@@ -33366,13 +33366,13 @@
         <v>0</v>
       </c>
       <c r="P66" s="7" t="n">
-        <v>4852080.3</v>
+        <v>11928823.02</v>
       </c>
       <c r="Q66" s="9" t="n">
-        <v>0.4067526437323236</v>
+        <v>0.4067</v>
       </c>
       <c r="R66" s="7" t="n">
-        <v>7076742.72</v>
+        <v>7076780.22</v>
       </c>
       <c r="S66" s="7" t="n">
         <v>0</v>
@@ -33650,13 +33650,13 @@
         <v>0</v>
       </c>
       <c r="P67" s="7" t="n">
-        <v>11551184.42</v>
+        <v>11551184.44</v>
       </c>
       <c r="Q67" s="9" t="n">
-        <v>0.9999999982685759</v>
+        <v>1</v>
       </c>
       <c r="R67" s="7" t="n">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="S67" s="7" t="n">
         <v>0</v>
@@ -33934,13 +33934,13 @@
         <v>0</v>
       </c>
       <c r="P68" s="7" t="n">
-        <v>41516316.78</v>
+        <v>44149151.5</v>
       </c>
       <c r="Q68" s="9" t="n">
-        <v>0.940364998407727</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="R68" s="7" t="n">
-        <v>2632834.72</v>
+        <v>2648192.01</v>
       </c>
       <c r="S68" s="7" t="n">
         <v>0</v>
@@ -34214,10 +34214,10 @@
         <v>0</v>
       </c>
       <c r="P69" s="7" t="n">
-        <v>1496414.32</v>
+        <v>1498793.43</v>
       </c>
       <c r="Q69" s="9" t="n">
-        <v>0.9984126498339402</v>
+        <v>0.9984000000000001</v>
       </c>
       <c r="R69" s="7" t="n">
         <v>2379.11</v>
@@ -34498,10 +34498,10 @@
         <v>0</v>
       </c>
       <c r="P70" s="7" t="n">
-        <v>64026819.34</v>
+        <v>89008310.65000001</v>
       </c>
       <c r="Q70" s="9" t="n">
-        <v>0.7193352943386079</v>
+        <v>0.7193000000000001</v>
       </c>
       <c r="R70" s="7" t="n">
         <v>24981491.31</v>
@@ -34778,10 +34778,10 @@
         <v>0</v>
       </c>
       <c r="P71" s="7" t="n">
-        <v>266299.23</v>
+        <v>8995898.050000001</v>
       </c>
       <c r="Q71" s="9" t="n">
-        <v>0.02960229523721647</v>
+        <v>0</v>
       </c>
       <c r="R71" s="7" t="n">
         <v>8729598.82</v>
@@ -35069,7 +35069,7 @@
         <v>18264452.89</v>
       </c>
       <c r="Q72" s="9" t="n">
-        <v>0.9999999999999998</v>
+        <v>1</v>
       </c>
       <c r="R72" s="7" t="n">
         <v>0</v>
@@ -35350,10 +35350,10 @@
         <v>0</v>
       </c>
       <c r="P73" s="7" t="n">
-        <v>88995375.53</v>
+        <v>90986818.17</v>
       </c>
       <c r="Q73" s="9" t="n">
-        <v>0.9781128444751286</v>
+        <v>0.9781</v>
       </c>
       <c r="R73" s="7" t="n">
         <v>1991442.64</v>
@@ -35634,10 +35634,10 @@
         <v>0</v>
       </c>
       <c r="P74" s="7" t="n">
-        <v>35196032.93</v>
+        <v>36880209</v>
       </c>
       <c r="Q74" s="9" t="n">
-        <v>0.9543338794527981</v>
+        <v>0.9543</v>
       </c>
       <c r="R74" s="7" t="n">
         <v>1684176.07</v>
@@ -35918,13 +35918,13 @@
         <v>0</v>
       </c>
       <c r="P75" s="7" t="n">
-        <v>19910338.67</v>
+        <v>20229149.79</v>
       </c>
       <c r="Q75" s="9" t="n">
-        <v>0.9842400138755413</v>
+        <v>0.9842</v>
       </c>
       <c r="R75" s="7" t="n">
-        <v>318811.12</v>
+        <v>318751.42</v>
       </c>
       <c r="S75" s="7" t="n">
         <v>0</v>
@@ -36202,10 +36202,10 @@
         <v>0</v>
       </c>
       <c r="P76" s="7" t="n">
-        <v>56828.03</v>
+        <v>2317778.22</v>
       </c>
       <c r="Q76" s="9" t="n">
-        <v>0.02451832082536352</v>
+        <v>0.0245</v>
       </c>
       <c r="R76" s="7" t="n">
         <v>2260950.19</v>
@@ -36482,13 +36482,13 @@
         <v>0</v>
       </c>
       <c r="P77" s="7" t="n">
-        <v>3552073.1</v>
+        <v>3552093.82</v>
       </c>
       <c r="Q77" s="9" t="n">
-        <v>0.9999941668207402</v>
+        <v>1</v>
       </c>
       <c r="R77" s="7" t="n">
-        <v>20.72</v>
+        <v>20.69</v>
       </c>
       <c r="S77" s="7" t="n">
         <v>0</v>
@@ -36762,7 +36762,7 @@
         <v>0</v>
       </c>
       <c r="P78" s="7" t="n">
-        <v>0</v>
+        <v>10134014.66</v>
       </c>
       <c r="Q78" s="9" t="n">
         <v>0</v>
@@ -37052,7 +37052,7 @@
         <v>1</v>
       </c>
       <c r="R79" s="7" t="n">
-        <v>0</v>
+        <v>-0.17</v>
       </c>
       <c r="S79" s="7" t="n">
         <v>0</v>
@@ -37334,10 +37334,10 @@
         <v>0</v>
       </c>
       <c r="P80" s="7" t="n">
-        <v>147280622.62</v>
+        <v>148784461.49</v>
       </c>
       <c r="Q80" s="9" t="n">
-        <v>0.9898925005007927</v>
+        <v>0.9899</v>
       </c>
       <c r="R80" s="7" t="n">
         <v>1503838.87</v>
@@ -37614,10 +37614,10 @@
         <v>0</v>
       </c>
       <c r="P81" s="7" t="n">
-        <v>12576165.07</v>
+        <v>22759968.59</v>
       </c>
       <c r="Q81" s="9" t="n">
-        <v>0.5525563455973117</v>
+        <v>0.5526</v>
       </c>
       <c r="R81" s="7" t="n">
         <v>10183803.52</v>
@@ -37902,10 +37902,10 @@
         <v>0</v>
       </c>
       <c r="P82" s="7" t="n">
-        <v>1940441.71</v>
+        <v>27739392.32</v>
       </c>
       <c r="Q82" s="9" t="n">
-        <v>0.06995256736756085</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="R82" s="7" t="n">
         <v>25798950.61</v>
@@ -38182,10 +38182,10 @@
         <v>0</v>
       </c>
       <c r="P83" s="7" t="n">
-        <v>5260332.26</v>
+        <v>5312585.57</v>
       </c>
       <c r="Q83" s="9" t="n">
-        <v>0.9901642412509883</v>
+        <v>0.9902</v>
       </c>
       <c r="R83" s="7" t="n">
         <v>52253.31</v>
@@ -38466,13 +38466,13 @@
         <v>0</v>
       </c>
       <c r="P84" s="7" t="n">
-        <v>5319860.7</v>
+        <v>5361446.28</v>
       </c>
       <c r="Q84" s="9" t="n">
-        <v>0.9922435891682567</v>
+        <v>0.9922</v>
       </c>
       <c r="R84" s="7" t="n">
-        <v>41585.58</v>
+        <v>41684.58</v>
       </c>
       <c r="S84" s="7" t="n">
         <v>0</v>
@@ -38746,13 +38746,13 @@
         <v>0</v>
       </c>
       <c r="P85" s="7" t="n">
-        <v>2867505.09</v>
+        <v>2994510.29</v>
       </c>
       <c r="Q85" s="9" t="n">
-        <v>0.9575873222329117</v>
+        <v>0.9577</v>
       </c>
       <c r="R85" s="7" t="n">
-        <v>127005.2</v>
+        <v>126804.97</v>
       </c>
       <c r="S85" s="7" t="n">
         <v>0</v>
@@ -39026,10 +39026,10 @@
         <v>0</v>
       </c>
       <c r="P86" s="7" t="n">
-        <v>8156656.13</v>
+        <v>8156656.19</v>
       </c>
       <c r="Q86" s="9" t="n">
-        <v>0.9999999926440444</v>
+        <v>1</v>
       </c>
       <c r="R86" s="7" t="n">
         <v>0.06</v>
@@ -39310,13 +39310,13 @@
         <v>0</v>
       </c>
       <c r="P87" s="7" t="n">
-        <v>7148655.62</v>
+        <v>7155724.39</v>
       </c>
       <c r="Q87" s="9" t="n">
-        <v>0.9990121517243065</v>
+        <v>0.9990000000000001</v>
       </c>
       <c r="R87" s="7" t="n">
-        <v>7068.77</v>
+        <v>7068.79</v>
       </c>
       <c r="S87" s="7" t="n">
         <v>0</v>
@@ -39598,13 +39598,13 @@
         <v>0</v>
       </c>
       <c r="P88" s="7" t="n">
-        <v>5991696.66</v>
+        <v>6765672.29</v>
       </c>
       <c r="Q88" s="9" t="n">
-        <v>0.8856025540663601</v>
+        <v>0.8856000000000001</v>
       </c>
       <c r="R88" s="7" t="n">
-        <v>773975.63</v>
+        <v>773975.71</v>
       </c>
       <c r="S88" s="7" t="n">
         <v>0</v>
@@ -39878,10 +39878,10 @@
         <v>0</v>
       </c>
       <c r="P89" s="7" t="n">
-        <v>137475.09</v>
+        <v>21672861.46</v>
       </c>
       <c r="Q89" s="9" t="n">
-        <v>0.006343190549790927</v>
+        <v>0.0063</v>
       </c>
       <c r="R89" s="7" t="n">
         <v>21535386.37</v>
@@ -40158,10 +40158,10 @@
         <v>0</v>
       </c>
       <c r="P90" s="7" t="n">
-        <v>31178236.21</v>
+        <v>32836774.76</v>
       </c>
       <c r="Q90" s="9" t="n">
-        <v>0.9494914295900844</v>
+        <v>0.9495</v>
       </c>
       <c r="R90" s="7" t="n">
         <v>1658538.55</v>
@@ -40438,7 +40438,7 @@
         <v>0</v>
       </c>
       <c r="P91" s="7" t="n">
-        <v>0</v>
+        <v>14144248.92</v>
       </c>
       <c r="Q91" s="9" t="n">
         <v>0</v>
@@ -40722,13 +40722,13 @@
         <v>0</v>
       </c>
       <c r="P92" s="7" t="n">
-        <v>1923627.24</v>
+        <v>1923627.23</v>
       </c>
       <c r="Q92" s="9" t="n">
-        <v>1.000000005198513</v>
+        <v>1</v>
       </c>
       <c r="R92" s="7" t="n">
-        <v>-0.01</v>
+        <v>-0.03</v>
       </c>
       <c r="S92" s="7" t="n">
         <v>0</v>
@@ -41006,10 +41006,10 @@
         <v>0</v>
       </c>
       <c r="P93" s="7" t="n">
-        <v>127835.64</v>
+        <v>16774604.06</v>
       </c>
       <c r="Q93" s="9" t="n">
-        <v>0.007620784344164126</v>
+        <v>0.0076</v>
       </c>
       <c r="R93" s="7" t="n">
         <v>16646768.42</v>
@@ -41290,7 +41290,7 @@
         <v>0</v>
       </c>
       <c r="P94" s="7" t="n">
-        <v>0</v>
+        <v>6784130.44</v>
       </c>
       <c r="Q94" s="9" t="n">
         <v>0</v>
@@ -41574,10 +41574,10 @@
         <v>0</v>
       </c>
       <c r="P95" s="7" t="n">
-        <v>30456294.33</v>
+        <v>30599999.01</v>
       </c>
       <c r="Q95" s="9" t="n">
-        <v>0.9953037684755141</v>
+        <v>0.9953</v>
       </c>
       <c r="R95" s="7" t="n">
         <v>143704.68</v>
@@ -41854,10 +41854,10 @@
         <v>0</v>
       </c>
       <c r="P96" s="7" t="n">
-        <v>264324.6</v>
+        <v>2394811.95</v>
       </c>
       <c r="Q96" s="9" t="n">
-        <v>0.1103738437583794</v>
+        <v>0.1104</v>
       </c>
       <c r="R96" s="7" t="n">
         <v>2130487.35</v>
@@ -42138,13 +42138,13 @@
         <v>0</v>
       </c>
       <c r="P97" s="7" t="n">
-        <v>26930984.01</v>
+        <v>26946699.36</v>
       </c>
       <c r="Q97" s="9" t="n">
-        <v>0.9994167987036167</v>
+        <v>0.9994</v>
       </c>
       <c r="R97" s="7" t="n">
-        <v>15715.35</v>
+        <v>15715.34</v>
       </c>
       <c r="S97" s="7" t="n">
         <v>0</v>
@@ -42422,10 +42422,10 @@
         <v>0</v>
       </c>
       <c r="P98" s="7" t="n">
-        <v>5996889.68</v>
+        <v>6014775.77</v>
       </c>
       <c r="Q98" s="9" t="n">
-        <v>0.9970263080979328</v>
+        <v>0.997</v>
       </c>
       <c r="R98" s="7" t="n">
         <v>17886.09</v>
@@ -42706,10 +42706,10 @@
         <v>0</v>
       </c>
       <c r="P99" s="7" t="n">
-        <v>3538001.16</v>
+        <v>3569195.39</v>
       </c>
       <c r="Q99" s="9" t="n">
-        <v>0.9912601506526095</v>
+        <v>0.9913</v>
       </c>
       <c r="R99" s="7" t="n">
         <v>31194.23</v>
@@ -42986,10 +42986,10 @@
         <v>0</v>
       </c>
       <c r="P100" s="7" t="n">
-        <v>2975297.32</v>
+        <v>2975474.34</v>
       </c>
       <c r="Q100" s="9" t="n">
-        <v>0.9999405069646813</v>
+        <v>0.9998999999999999</v>
       </c>
       <c r="R100" s="7" t="n">
         <v>177.02</v>
@@ -43546,10 +43546,10 @@
         <v>0</v>
       </c>
       <c r="P102" s="7" t="n">
-        <v>1932548.63</v>
+        <v>1988555.07</v>
       </c>
       <c r="Q102" s="9" t="n">
-        <v>0.9718356102654981</v>
+        <v>0.9718000000000001</v>
       </c>
       <c r="R102" s="7" t="n">
         <v>56006.44</v>
@@ -43826,13 +43826,13 @@
         <v>0</v>
       </c>
       <c r="P103" s="7" t="n">
-        <v>1678310.19</v>
+        <v>1690234.37</v>
       </c>
       <c r="Q103" s="9" t="n">
-        <v>0.9929452505453428</v>
+        <v>0.9931</v>
       </c>
       <c r="R103" s="7" t="n">
-        <v>11924.18</v>
+        <v>11624.18</v>
       </c>
       <c r="S103" s="7" t="n">
         <v>0</v>
@@ -44110,13 +44110,13 @@
         <v>0</v>
       </c>
       <c r="P104" s="7" t="n">
-        <v>1612016.33</v>
+        <v>1612154.63</v>
       </c>
       <c r="Q104" s="9" t="n">
-        <v>0.9999142141842808</v>
+        <v>0.9998999999999999</v>
       </c>
       <c r="R104" s="7" t="n">
-        <v>138.3</v>
+        <v>129.78</v>
       </c>
       <c r="S104" s="7" t="n">
         <v>0</v>
@@ -44394,13 +44394,13 @@
         <v>0</v>
       </c>
       <c r="P105" s="7" t="n">
-        <v>25102277.93</v>
+        <v>25179808.67</v>
       </c>
       <c r="Q105" s="9" t="n">
-        <v>0.9969209162382409</v>
+        <v>0.9969</v>
       </c>
       <c r="R105" s="7" t="n">
-        <v>77530.74000000001</v>
+        <v>77530.64</v>
       </c>
       <c r="S105" s="7" t="n">
         <v>0</v>
@@ -44681,10 +44681,10 @@
         <v>666913.6800000001</v>
       </c>
       <c r="Q106" s="9" t="n">
-        <v>1</v>
+        <v>0.8991</v>
       </c>
       <c r="R106" s="7" t="n">
-        <v>0</v>
+        <v>67272.37</v>
       </c>
       <c r="S106" s="7" t="n">
         <v>0</v>
@@ -44962,10 +44962,10 @@
         <v>0</v>
       </c>
       <c r="P107" s="7" t="n">
-        <v>1006235.15</v>
+        <v>1052239.53</v>
       </c>
       <c r="Q107" s="9" t="n">
-        <v>0.9562795554734577</v>
+        <v>0.9562999999999999</v>
       </c>
       <c r="R107" s="7" t="n">
         <v>46004.38</v>
@@ -45246,10 +45246,10 @@
         <v>0</v>
       </c>
       <c r="P108" s="7" t="n">
-        <v>13180256.4</v>
+        <v>14782911.98</v>
       </c>
       <c r="Q108" s="9" t="n">
-        <v>0.8915872879329693</v>
+        <v>0.8915999999999999</v>
       </c>
       <c r="R108" s="7" t="n">
         <v>1602655.58</v>
@@ -45533,7 +45533,7 @@
         <v>62980000</v>
       </c>
       <c r="Q109" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R109" s="7" t="n">
         <v>0</v>
@@ -45814,13 +45814,13 @@
         <v>0</v>
       </c>
       <c r="P110" s="7" t="n">
-        <v>12888606.56</v>
+        <v>13554947.83</v>
       </c>
       <c r="Q110" s="9" t="n">
-        <v>0.9508414729177163</v>
+        <v>0.9508</v>
       </c>
       <c r="R110" s="7" t="n">
-        <v>666341.27</v>
+        <v>666441.27</v>
       </c>
       <c r="S110" s="7" t="n">
         <v>0</v>
@@ -46098,10 +46098,10 @@
         <v>0</v>
       </c>
       <c r="P111" s="7" t="n">
-        <v>296101.87</v>
+        <v>13677862.32</v>
       </c>
       <c r="Q111" s="9" t="n">
-        <v>0.02164825636291388</v>
+        <v>0.0216</v>
       </c>
       <c r="R111" s="7" t="n">
         <v>13381760.45</v>
@@ -46382,10 +46382,10 @@
         <v>0</v>
       </c>
       <c r="P112" s="7" t="n">
-        <v>54872063.4</v>
+        <v>56185153.92</v>
       </c>
       <c r="Q112" s="9" t="n">
-        <v>0.9766292262566429</v>
+        <v>0.9765999999999999</v>
       </c>
       <c r="R112" s="7" t="n">
         <v>1313090.52</v>
@@ -46666,10 +46666,10 @@
         <v>0</v>
       </c>
       <c r="P113" s="7" t="n">
-        <v>13048536.54</v>
+        <v>16880240</v>
       </c>
       <c r="Q113" s="9" t="n">
-        <v>0.7730065769207074</v>
+        <v>0.773</v>
       </c>
       <c r="R113" s="7" t="n">
         <v>3831703.46</v>
@@ -46950,13 +46950,13 @@
         <v>0</v>
       </c>
       <c r="P114" s="7" t="n">
-        <v>5728240.72</v>
+        <v>6519257.05</v>
       </c>
       <c r="Q114" s="9" t="n">
-        <v>0.8786646509052747</v>
+        <v>0.8787</v>
       </c>
       <c r="R114" s="7" t="n">
-        <v>791016.33</v>
+        <v>791016.1899999999</v>
       </c>
       <c r="S114" s="7" t="n">
         <v>0</v>
@@ -47234,13 +47234,13 @@
         <v>0</v>
       </c>
       <c r="P115" s="7" t="n">
-        <v>45858219.18</v>
+        <v>48302952.43</v>
       </c>
       <c r="Q115" s="9" t="n">
-        <v>0.9493874985479848</v>
+        <v>0.9493</v>
       </c>
       <c r="R115" s="7" t="n">
-        <v>2444733.25</v>
+        <v>2449729.13</v>
       </c>
       <c r="S115" s="7" t="n">
         <v>0</v>
@@ -47518,10 +47518,10 @@
         <v>0</v>
       </c>
       <c r="P116" s="7" t="n">
-        <v>255684.47</v>
+        <v>3615856.15</v>
       </c>
       <c r="Q116" s="9" t="n">
-        <v>0.07071201380619081</v>
+        <v>0.0707</v>
       </c>
       <c r="R116" s="7" t="n">
         <v>3360171.68</v>
@@ -47802,10 +47802,10 @@
         <v>0</v>
       </c>
       <c r="P117" s="7" t="n">
-        <v>8398407.23</v>
+        <v>24165422.12</v>
       </c>
       <c r="Q117" s="9" t="n">
-        <v>0.3475381968622528</v>
+        <v>0.3475</v>
       </c>
       <c r="R117" s="7" t="n">
         <v>15767014.89</v>
@@ -48086,13 +48086,13 @@
         <v>0</v>
       </c>
       <c r="P118" s="7" t="n">
-        <v>14985593.44</v>
+        <v>14995089.28</v>
       </c>
       <c r="Q118" s="9" t="n">
-        <v>0.9993667366814106</v>
+        <v>0.9994</v>
       </c>
       <c r="R118" s="7" t="n">
-        <v>9495.84</v>
+        <v>9530.83</v>
       </c>
       <c r="S118" s="7" t="n">
         <v>0</v>
@@ -48370,13 +48370,13 @@
         <v>0</v>
       </c>
       <c r="P119" s="7" t="n">
-        <v>14660281.99</v>
+        <v>15078640.21</v>
       </c>
       <c r="Q119" s="9" t="n">
-        <v>0.9722549106435638</v>
+        <v>0.9723000000000001</v>
       </c>
       <c r="R119" s="7" t="n">
-        <v>418358.22</v>
+        <v>418357.84</v>
       </c>
       <c r="S119" s="7" t="n">
         <v>0</v>
@@ -48654,10 +48654,10 @@
         <v>0</v>
       </c>
       <c r="P120" s="7" t="n">
-        <v>21925638.52</v>
+        <v>24590858.27</v>
       </c>
       <c r="Q120" s="9" t="n">
-        <v>0.8916174571567731</v>
+        <v>0.8915999999999999</v>
       </c>
       <c r="R120" s="7" t="n">
         <v>2665219.75</v>
@@ -48938,10 +48938,10 @@
         <v>0</v>
       </c>
       <c r="P121" s="7" t="n">
-        <v>9082408.67</v>
+        <v>16932981.45</v>
       </c>
       <c r="Q121" s="9" t="n">
-        <v>0.5363738628556755</v>
+        <v>0.5364</v>
       </c>
       <c r="R121" s="7" t="n">
         <v>7850572.78</v>

</xml_diff>

<commit_message>
Atualiza base e consolidado de medições
</commit_message>
<xml_diff>
--- a/MEDIÇÕES_CONSOLIDADO.xlsx
+++ b/MEDIÇÕES_CONSOLIDADO.xlsx
@@ -9586,7 +9586,7 @@
         <v>2715707.77</v>
       </c>
       <c r="N32" s="7" t="n">
-        <v>0</v>
+        <v>905475.02</v>
       </c>
       <c r="O32" s="7" t="n">
         <v>22825141.32</v>
@@ -9778,7 +9778,7 @@
         <v>392686.6</v>
       </c>
       <c r="BZ32" s="7" t="n">
-        <v>0</v>
+        <v>905475.02</v>
       </c>
       <c r="CA32" s="7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualiza arquivos gerados de medicoes
</commit_message>
<xml_diff>
--- a/MEDIÇÕES_CONSOLIDADO.xlsx
+++ b/MEDIÇÕES_CONSOLIDADO.xlsx
@@ -4489,10 +4489,10 @@
         </is>
       </c>
       <c r="M14" s="7" t="n">
-        <v>0</v>
+        <v>842876.36</v>
       </c>
       <c r="N14" s="7" t="n">
-        <v>0</v>
+        <v>1284711.9</v>
       </c>
       <c r="O14" s="7" t="n">
         <v>7848019.53</v>
@@ -4681,10 +4681,10 @@
         <v>0</v>
       </c>
       <c r="BY14" s="7" t="n">
-        <v>0</v>
+        <v>842876.36</v>
       </c>
       <c r="BZ14" s="7" t="n">
-        <v>0</v>
+        <v>1284711.9</v>
       </c>
       <c r="CA14" s="7" t="n">
         <v>0</v>
@@ -15236,7 +15236,7 @@
         <v>55173009.47</v>
       </c>
       <c r="N52" s="7" t="n">
-        <v>1537890.45</v>
+        <v>5219382.56</v>
       </c>
       <c r="O52" s="7" t="n">
         <v>74609626.42</v>
@@ -15431,7 +15431,7 @@
         <v>1537890.45</v>
       </c>
       <c r="CA52" s="7" t="n">
-        <v>0</v>
+        <v>3681492.11</v>
       </c>
       <c r="CB52" s="7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Atualiza medições processadas e arquivos de comissões
</commit_message>
<xml_diff>
--- a/MEDIÇÕES_CONSOLIDADO.xlsx
+++ b/MEDIÇÕES_CONSOLIDADO.xlsx
@@ -4489,10 +4489,10 @@
         </is>
       </c>
       <c r="M14" s="7" t="n">
-        <v>842876.36</v>
+        <v>0</v>
       </c>
       <c r="N14" s="7" t="n">
-        <v>1284711.9</v>
+        <v>0</v>
       </c>
       <c r="O14" s="7" t="n">
         <v>7848019.53</v>
@@ -4681,10 +4681,10 @@
         <v>0</v>
       </c>
       <c r="BY14" s="7" t="n">
-        <v>842876.36</v>
+        <v>0</v>
       </c>
       <c r="BZ14" s="7" t="n">
-        <v>1284711.9</v>
+        <v>0</v>
       </c>
       <c r="CA14" s="7" t="n">
         <v>0</v>
@@ -5058,7 +5058,7 @@
         <v>10584628.26</v>
       </c>
       <c r="N16" s="7" t="n">
-        <v>519586.74</v>
+        <v>1199631.94</v>
       </c>
       <c r="O16" s="7" t="n">
         <v>48872552.26</v>
@@ -5253,7 +5253,7 @@
         <v>519586.74</v>
       </c>
       <c r="CA16" s="7" t="n">
-        <v>0</v>
+        <v>680045.2</v>
       </c>
       <c r="CB16" s="7" t="n">
         <v>0</v>
@@ -46348,7 +46348,7 @@
         <v>710964.03</v>
       </c>
       <c r="O109" s="7" t="n">
-        <v>0</v>
+        <v>294655.66</v>
       </c>
       <c r="P109" s="7" t="n">
         <v>13554947.83</v>
@@ -46486,7 +46486,7 @@
         <v>712517.77</v>
       </c>
       <c r="BI109" s="7" t="n">
-        <v>528677.09</v>
+        <v>528577.09</v>
       </c>
       <c r="BJ109" s="7" t="n">
         <v>598849.04</v>
@@ -46540,7 +46540,7 @@
         <v>0</v>
       </c>
       <c r="CA109" s="7" t="n">
-        <v>0</v>
+        <v>294655.66</v>
       </c>
       <c r="CB109" s="7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Processa medições e atualiza planilhas
</commit_message>
<xml_diff>
--- a/MEDIÇÕES_CONSOLIDADO.xlsx
+++ b/MEDIÇÕES_CONSOLIDADO.xlsx
@@ -3900,7 +3900,11 @@
           <t>EXECUÇÃO</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>ISADORA ROSALINO</t>
+        </is>
+      </c>
       <c r="J12" s="10" t="inlineStr">
         <is>
           <t>NT</t>
@@ -5592,7 +5596,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>IGOR MARTINS</t>
+          <t>JAQUELINE PASTÓRIO</t>
         </is>
       </c>
       <c r="J18" s="8" t="inlineStr">
@@ -16883,8 +16887,16 @@
           <t>NÃO CONCLUÍDA</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr"/>
-      <c r="J3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>CARLOS FERNANDES</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>ANDERSON / OTAVIO FEITOSA</t>
+        </is>
+      </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
           <t>BX</t>
@@ -17163,8 +17175,16 @@
           <t>NÃO CONCLUÍDA</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr"/>
-      <c r="J4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>CARLOS FERNANDES</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>ANDERSON / OTAVIO FEITOSA</t>
+        </is>
+      </c>
       <c r="K4" s="11" t="inlineStr">
         <is>
           <t>BX</t>
@@ -17450,7 +17470,7 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>NICHOLAS TAVARES / OTAVIO FEITOSA</t>
+          <t>ANDERSON / OTAVIO FEITOSA</t>
         </is>
       </c>
       <c r="K5" s="11" t="inlineStr">
@@ -19711,8 +19731,16 @@
           <t>CONCLUÍDA</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr"/>
-      <c r="J13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>CARLOS FERNANDES</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>ANDERSON / OTAVIO FEITOSA</t>
+        </is>
+      </c>
       <c r="K13" s="8" t="inlineStr">
         <is>
           <t>SL</t>
@@ -23394,7 +23422,7 @@
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>NICHOLAS TAVARES / OTAVIO FEITOSA</t>
+          <t>ANDERSON / OTAVIO FEITOSA</t>
         </is>
       </c>
       <c r="K26" s="11" t="inlineStr">
@@ -29881,10 +29909,14 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>GISELLE G. FONSECA</t>
-        </is>
-      </c>
-      <c r="J49" s="4" t="inlineStr"/>
+          <t>CARLOS FERNANDES</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>ANDERSON / OTAVIO FEITOSA</t>
+        </is>
+      </c>
       <c r="K49" s="11" t="inlineStr">
         <is>
           <t>BX</t>
@@ -31586,7 +31618,7 @@
       </c>
       <c r="J55" s="4" t="inlineStr">
         <is>
-          <t>HIGOR GAMA / OTAVIO FEITOSA</t>
+          <t>HIGOR GAMA / JOAO JOSE</t>
         </is>
       </c>
       <c r="K55" s="8" t="inlineStr">
@@ -33018,7 +33050,7 @@
       </c>
       <c r="J60" s="4" t="inlineStr">
         <is>
-          <t>NICHOLAS TAVARES / ARLINDO BASILIO</t>
+          <t>ANDERSON / OTAVIO FEITOSA</t>
         </is>
       </c>
       <c r="K60" s="11" t="inlineStr">
@@ -33306,7 +33338,7 @@
       </c>
       <c r="J61" s="4" t="inlineStr">
         <is>
-          <t>ARLINDO BASILIO / OTAVIO FEITOSA</t>
+          <t>ANDERSON / OTAVIO FEITOSA</t>
         </is>
       </c>
       <c r="K61" s="11" t="inlineStr">
@@ -33878,7 +33910,7 @@
       </c>
       <c r="J63" s="4" t="inlineStr">
         <is>
-          <t>LUCIANA POSTIÇO / OTAVIO FEITOSA</t>
+          <t>HIGOR GAMA / JOAO JOSE</t>
         </is>
       </c>
       <c r="K63" s="11" t="inlineStr">
@@ -38680,7 +38712,7 @@
       </c>
       <c r="J80" s="4" t="inlineStr">
         <is>
-          <t>NICHOLAS TAVARES / OSVALDO NETO</t>
+          <t>ANDERSON / OTAVIO FEITOSA</t>
         </is>
       </c>
       <c r="K80" s="11" t="inlineStr">
@@ -39243,12 +39275,12 @@
       </c>
       <c r="I82" s="4" t="inlineStr">
         <is>
-          <t>JEHNIFFER PIRES</t>
+          <t>GISELLE G. FONSECA</t>
         </is>
       </c>
       <c r="J82" s="4" t="inlineStr">
         <is>
-          <t>LUCIANA POSTIÇO / ARLINDO BASILIO</t>
+          <t>HIGOR GAMA / JOAO JOSE</t>
         </is>
       </c>
       <c r="K82" s="8" t="inlineStr">
@@ -50257,7 +50289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B44"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50395,394 +50427,346 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>330018/000424/2021</t>
+          <t>170026/001865/2021</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ALBERTO COUTO ALVES - BRASIL LTDA.</t>
+          <t>SANTA LUZIA ENGENHARIA E CONSTRUCOES LTDA</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>330018/000423/2021</t>
+          <t>330018/000235/2020</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ALBERTO COUTO ALVES - BRASIL LTDA.</t>
+          <t>CRATER CONSTRUÇÕES LTDA.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>170026/001178/2021</t>
+          <t>170026/001229/2022</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>COLÔNIA ARQUITETURA E CONSTRUÇÃO EIRELI EPP</t>
+          <t>BARRA NOVA ENGENHARIA LTDA</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>170026/001865/2021</t>
+          <t>170026/001230/2022</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SANTA LUZIA ENGENHARIA E CONSTRUCOES LTDA</t>
+          <t>RIVALL ENGENHARIA LTDA</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>330018/000235/2020</t>
+          <t>170026/001231/2022</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CRATER CONSTRUÇÕES LTDA.</t>
+          <t>ECONORTE, MEIO AMBIENTE, INFRAESTRUTURA E SERVIÇOS LTDA</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>170026/001229/2022</t>
+          <t>170026/002388/2021</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BARRA NOVA ENGENHARIA LTDA</t>
+          <t>WTE ENGENHARIA EIRELI</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>170026/001230/2022</t>
+          <t>330018/000712/2021</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>RIVALL ENGENHARIA LTDA</t>
+          <t>SEEL SERVICOS ESPECIAIS DE ENGENHARIA LTDA</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>170026/001231/2022</t>
+          <t>330018/001017/2021</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ECONORTE, MEIO AMBIENTE, INFRAESTRUTURA E SERVIÇOS LTDA</t>
+          <t>NOVACAP ENGENHARIA, INDUSTRIS E COMERCIO LTDA</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>170026/002388/2021</t>
+          <t>170026/000549/2022</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>WTE ENGENHARIA EIRELI</t>
+          <t>BARRA NOVA ENGENHARIA LTDA</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>330001/001238/2025</t>
+          <t>170026/001072/2022</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ENEX CONSTRUÇÕES LTDA</t>
+          <t>COORDENA COORDENAÇÃO DE PROJETOS LTDA</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>330018/000712/2021</t>
+          <t>170026/000548/2022</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SEEL SERVICOS ESPECIAIS DE ENGENHARIA LTDA</t>
+          <t>ENGE PRAT ENGENHARIA E SERVICOS LTDA.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>330018/001017/2021</t>
+          <t>170026/000537/2022</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>NOVACAP ENGENHARIA, INDUSTRIS E COMERCIO LTDA</t>
+          <t>ERWIL CONSTRUÇÕES LTDA</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>170026/000549/2022</t>
+          <t>170026/000545/2022</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BARRA NOVA ENGENHARIA LTDA</t>
+          <t>GEOLOGUS ENGENHARIA LTDA</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>170026/001072/2022</t>
+          <t>170026/000539/2022</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>COORDENA COORDENAÇÃO DE PROJETOS LTDA</t>
+          <t>CONSTRUTORA SOLIDUM  LTDA</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>170026/000548/2022</t>
+          <t>330018/000580/2022</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ENGE PRAT ENGENHARIA E SERVICOS LTDA.</t>
+          <t>MEDEIROS E MEDEIROS CIVIL E MONTAGEM LTDA-ME</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>170026/000537/2022</t>
+          <t>170026/001303/2020</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ERWIL CONSTRUÇÕES LTDA</t>
+          <t>WTE ENGENHARIA EIRELI</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>170026/000545/2022</t>
+          <t>170026/001868/2021</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>GEOLOGUS ENGENHARIA LTDA</t>
+          <t>WTE ENGENHARIA EIRELI</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>170026/000539/2022</t>
+          <t>330018/001037/2021</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CONSTRUTORA SOLIDUM  LTDA</t>
+          <t>COMAL CONSTRUTORA LTDA</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>330018/000580/2022</t>
+          <t>170026/002018/2021</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MEDEIROS E MEDEIROS CIVIL E MONTAGEM LTDA-ME</t>
+          <t>DE SÁ CONSTRUÇÕES E SERVIÇOS LTDA</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>170026/001303/2020</t>
+          <t>170026/000379/2022</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>WTE ENGENHARIA EIRELI</t>
+          <t>GEOMECÂNICA S/A TECNOLOGIA DE SOLOS ROCHAS E MATERIAIS LTDA</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>170026/001868/2021</t>
+          <t>e-17/026/1892/2019-2</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>WTE ENGENHARIA EIRELI</t>
+          <t>FAB MIX CONCRETOS LTDA</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>330018/001037/2021</t>
+          <t>e-17/026/1892/2019-1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>COMAL CONSTRUTORA LTDA</t>
+          <t>METALURGICA BIG FARM LTDA</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>170026/002018/2021</t>
+          <t>170026/001763/2021</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DE SÁ CONSTRUÇÕES E SERVIÇOS LTDA</t>
+          <t>COMPASS - BUILD CONTROL LTDA</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>170026/000379/2022</t>
+          <t>E-17/001/81/2013</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>GEOMECÂNICA S/A TECNOLOGIA DE SOLOS ROCHAS E MATERIAIS LTDA</t>
+          <t>SEVEME INDUSTRIAS METALURGICAS S.A.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>e-17/026/1892/2019-2</t>
+          <t>330001/000434/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>FAB MIX CONCRETOS LTDA</t>
+          <t>Não existe na tabela Contratadas</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>e-17/026/1892/2019-1</t>
+          <t>330001/000113/2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>METALURGICA BIG FARM LTDA</t>
+          <t>Não existe na tabela Contratadas</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>170026/001763/2021</t>
+          <t>330001/001152/2025</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>COMPASS - BUILD CONTROL LTDA</t>
+          <t>Não existe na tabela Contratadas</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>E-17/001/81/2013</t>
+          <t>330018/000559/2022</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SEVEME INDUSTRIAS METALURGICAS S.A.</t>
+          <t>CONSTRUTORA METROPOLITANA S A</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>330001/000434/2026</t>
+          <t>330018/000221/2022</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
-        <is>
-          <t>Não existe na tabela Contratadas</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>330001/000113/2026</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Não existe na tabela Contratadas</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>330001/001152/2025</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Não existe na tabela Contratadas</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>330018/000559/2022</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>CONSTRUTORA METROPOLITANA S A</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>330018/000221/2022</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
         <is>
           <t>CONSTRUTORA LYTORANEA S A</t>
         </is>

</xml_diff>